<commit_message>
rearranged pages and added info
</commit_message>
<xml_diff>
--- a/codebook/codebook_votations.xlsx
+++ b/codebook/codebook_votations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\wd-poku\codebook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{631A0E06-1D15-4C38-89B4-AC73DAF4FB01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E74B565F-59B6-4725-8091-BA5066C1791A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{FA9B73F8-4F5D-4EB7-91DE-D73A293948DC}"/>
+    <workbookView xWindow="-8868" yWindow="14412" windowWidth="23256" windowHeight="13896" xr2:uid="{FA9B73F8-4F5D-4EB7-91DE-D73A293948DC}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -252,9 +252,6 @@
     <t>Number of eligible voters.</t>
   </si>
   <si>
-    <t>Number of valid votes.</t>
-  </si>
-  <si>
     <t>Available on the Swiss and cantonal level. For voting proposals on the federal level: only true, if gebietAusgezaehlt and vorlageBeendet is true for all cantons</t>
   </si>
   <si>
@@ -378,18 +375,12 @@
     <t>Number of fully counted municipalities in a given geographical unit.</t>
   </si>
   <si>
-    <t>Number of fully counted districts in a given geographical unit..</t>
-  </si>
-  <si>
     <t>see also https://bfspoku.github.io/wd-poku/geometries.html</t>
   </si>
   <si>
     <t>Parent identifier for the higher level geographical unit.</t>
   </si>
   <si>
-    <t xml:space="preserve">Indicates if the cantonal votes (staende) are relevant for the results of the vote. Generally true if a double majority is required for the proposal to be accepted. Also used for the deciding question. </t>
-  </si>
-  <si>
     <t xml:space="preserve">Display order of the proposal. </t>
   </si>
   <si>
@@ -405,9 +396,6 @@
     <t>Total number of districts in a given geographical unit.</t>
   </si>
   <si>
-    <t>Might be renamed in the future</t>
-  </si>
-  <si>
     <t>Only available on the canton level or higher and used only in the unharmonized files (sd-t-17-02-YYMMDD-eidgAbstimmung-o.json)</t>
   </si>
   <si>
@@ -466,6 +454,18 @@
   </si>
   <si>
     <t>Indicates if the counting process for a given proposal has ended and the result has been confirmed by the cantonal authority.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Indicates if the cantonal votes (staende) are relevant for the results of the vote. Generally true if a double majority is required for the proposal to be accepted. </t>
+  </si>
+  <si>
+    <t>Also used for the deciding question even though  the deciding question does not require a double majority. Might be renamed in the future</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Number of valid votes. In most cases, the number of valid votes on the federal level consists of the sum of yes and no votes. In the case of connected proposals, the "votes without response" (stimmen ohne Antwort) are also added to the number of valid ballots. </t>
+  </si>
+  <si>
+    <t>Number of fully counted districts in a given geographical unit.</t>
   </si>
 </sst>
 </file>
@@ -912,7 +912,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C2" t="s">
         <v>55</v>
@@ -929,7 +929,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C3" t="s">
         <v>56</v>
@@ -943,7 +943,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C4" t="s">
         <v>57</v>
@@ -957,7 +957,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C5" t="s">
         <v>58</v>
@@ -971,7 +971,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C6" t="s">
         <v>55</v>
@@ -988,7 +988,7 @@
         <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C7" t="s">
         <v>61</v>
@@ -1002,13 +1002,13 @@
         <v>12</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>58</v>
       </c>
       <c r="E8" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
@@ -1019,7 +1019,7 @@
         <v>14</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C9" s="6" t="s">
         <v>58</v>
@@ -1039,7 +1039,7 @@
         <v>62</v>
       </c>
       <c r="E10" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
@@ -1050,7 +1050,7 @@
         <v>16</v>
       </c>
       <c r="B11" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C11" t="s">
         <v>57</v>
@@ -1064,7 +1064,7 @@
         <v>17</v>
       </c>
       <c r="B12" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C12" s="6" t="s">
         <v>13</v>
@@ -1078,13 +1078,13 @@
         <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E13" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>
@@ -1095,13 +1095,13 @@
         <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>57</v>
       </c>
       <c r="E14" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="6"/>
@@ -1112,7 +1112,7 @@
         <v>20</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C15" s="6" t="s">
         <v>58</v>
@@ -1126,7 +1126,7 @@
         <v>21</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>58</v>
@@ -1140,13 +1140,13 @@
         <v>24</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="C17" s="6" t="s">
         <v>62</v>
       </c>
       <c r="E17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
@@ -1157,13 +1157,13 @@
         <v>22</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>62</v>
       </c>
       <c r="E18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
@@ -1174,10 +1174,10 @@
         <v>25</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
@@ -1188,13 +1188,13 @@
         <v>26</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>13</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
@@ -1205,13 +1205,13 @@
         <v>27</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>63</v>
       </c>
       <c r="E21" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
@@ -1222,7 +1222,7 @@
         <v>28</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>64</v>
@@ -1231,18 +1231,18 @@
       <c r="H22" s="6"/>
       <c r="I22" s="6"/>
     </row>
-    <row r="23" spans="1:9" ht="71.25" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" ht="57" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>29</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>62</v>
       </c>
       <c r="E23" t="s">
-        <v>122</v>
+        <v>140</v>
       </c>
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
@@ -1253,7 +1253,7 @@
         <v>30</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>61</v>
@@ -1267,7 +1267,7 @@
         <v>31</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>63</v>
@@ -1281,7 +1281,7 @@
         <v>32</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>63</v>
@@ -1295,7 +1295,7 @@
         <v>33</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>63</v>
@@ -1309,7 +1309,7 @@
         <v>34</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C28" s="6" t="s">
         <v>63</v>
@@ -1323,7 +1323,7 @@
         <v>35</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>63</v>
@@ -1337,7 +1337,7 @@
         <v>36</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>63</v>
@@ -1351,7 +1351,7 @@
         <v>51</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>57</v>
@@ -1363,7 +1363,7 @@
         <v>52</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>57</v>
@@ -1377,13 +1377,13 @@
         <v>53</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>57</v>
       </c>
       <c r="E33" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="G33" s="6"/>
       <c r="H33" s="6"/>
@@ -1394,13 +1394,13 @@
         <v>66</v>
       </c>
       <c r="B34" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E34" t="s">
         <v>75</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="E34" t="s">
-        <v>76</v>
       </c>
       <c r="G34" s="6"/>
       <c r="H34" s="6"/>
@@ -1411,13 +1411,13 @@
         <v>54</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>58</v>
       </c>
       <c r="E35" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G35" s="6"/>
       <c r="H35" s="6"/>
@@ -1428,7 +1428,7 @@
         <v>37</v>
       </c>
       <c r="B36" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>61</v>
@@ -1442,13 +1442,13 @@
         <v>38</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E37" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G37" s="6"/>
       <c r="H37" s="6"/>
@@ -1465,7 +1465,7 @@
         <v>13</v>
       </c>
       <c r="E38" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="G38" s="6"/>
       <c r="H38" s="6"/>
@@ -1476,13 +1476,13 @@
         <v>40</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>113</v>
+        <v>142</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E39" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="G39" s="6"/>
       <c r="H39" s="6"/>
@@ -1493,13 +1493,13 @@
         <v>41</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C40" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E40" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="G40" s="6"/>
       <c r="H40" s="6"/>
@@ -1510,13 +1510,13 @@
         <v>42</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C41" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E41" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="G41" s="6"/>
       <c r="H41" s="6"/>
@@ -1527,13 +1527,13 @@
         <v>43</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C42" s="6" t="s">
         <v>13</v>
       </c>
       <c r="E42" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="G42" s="6"/>
       <c r="H42" s="6"/>
@@ -1544,7 +1544,7 @@
         <v>5</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C43" s="6" t="s">
         <v>62</v>
@@ -1558,7 +1558,7 @@
         <v>44</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="C44" s="6" t="s">
         <v>65</v>
@@ -1572,7 +1572,7 @@
         <v>45</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="C45" s="6" t="s">
         <v>63</v>
@@ -1586,7 +1586,7 @@
         <v>46</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C46" s="6" t="s">
         <v>63</v>
@@ -1600,7 +1600,7 @@
         <v>47</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>65</v>
@@ -1637,12 +1637,12 @@
       <c r="H49" s="6"/>
       <c r="I49" s="6"/>
     </row>
-    <row r="50" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:10" ht="85.5" x14ac:dyDescent="0.2">
       <c r="A50" s="5" t="s">
         <v>50</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>71</v>
+        <v>141</v>
       </c>
       <c r="C50" s="6" t="s">
         <v>63</v>
@@ -1656,13 +1656,13 @@
         <v>23</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="C51" s="6" t="s">
         <v>57</v>
       </c>
       <c r="E51" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G51" s="6"/>
       <c r="H51" s="6"/>
@@ -1671,16 +1671,16 @@
     </row>
     <row r="52" spans="1:10" ht="15" x14ac:dyDescent="0.2">
       <c r="A52" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>58</v>
       </c>
       <c r="E52" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G52" s="6"/>
       <c r="H52" s="6"/>
@@ -1689,16 +1689,16 @@
     </row>
     <row r="53" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A53" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C53" s="6" t="s">
         <v>61</v>
       </c>
       <c r="E53" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G53" s="6"/>
       <c r="H53" s="6"/>
@@ -1707,16 +1707,16 @@
     </row>
     <row r="54" spans="1:10" ht="15" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B54" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C54" s="6" t="s">
         <v>58</v>
       </c>
       <c r="E54" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G54" s="6"/>
       <c r="H54" s="6"/>
@@ -1725,16 +1725,16 @@
     </row>
     <row r="55" spans="1:10" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C55" s="6" t="s">
         <v>61</v>
       </c>
       <c r="E55" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G55" s="6"/>
       <c r="H55" s="6"/>

</xml_diff>